<commit_message>
updated real valued SPICE sims for RF front end
</commit_message>
<xml_diff>
--- a/docs/2026-27-TVR/hardware/Telemetry-GND-Station/Documentation and Design Docs/Telemetry_GND_Station_Component_Selection.xlsx
+++ b/docs/2026-27-TVR/hardware/Telemetry-GND-Station/Documentation and Design Docs/Telemetry_GND_Station_Component_Selection.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\annie\Documents\UBC Rocket\Official Git\docs\docs\2026-27-TVR\hardware\Telemetry-GND-Station\Documentation and Design Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226F4B8B-8BCA-4700-AD1D-4A6C5EA58AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E3A2BB-868E-4A03-860D-E39F3E561E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ECEF2206-FE18-4489-9125-25D7FC7EFA54}"/>
+    <workbookView xWindow="1808" yWindow="3472" windowWidth="11677" windowHeight="9308" firstSheet="3" activeTab="5" xr2:uid="{ECEF2206-FE18-4489-9125-25D7FC7EFA54}"/>
   </bookViews>
   <sheets>
     <sheet name="Design Requirements" sheetId="1" r:id="rId1"/>
     <sheet name="Transciever IC " sheetId="3" r:id="rId2"/>
     <sheet name="Power Amplifier " sheetId="2" r:id="rId3"/>
-    <sheet name="Switches" sheetId="6" r:id="rId4"/>
-    <sheet name="Crystal" sheetId="4" r:id="rId5"/>
-    <sheet name="Filter" sheetId="5" r:id="rId6"/>
-    <sheet name="Matching" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId4"/>
+    <sheet name="Switches" sheetId="6" r:id="rId5"/>
+    <sheet name="Crystal" sheetId="4" r:id="rId6"/>
+    <sheet name="Filter" sheetId="5" r:id="rId7"/>
+    <sheet name="Matching" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -436,30 +437,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1223,18 +1222,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
       <c r="H2" t="s">
         <v>5</v>
       </c>
@@ -1405,18 +1404,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
@@ -1597,27 +1596,27 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
@@ -1645,6 +1644,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A32B04D4-73ED-42E1-B3D1-A53A8E3333E4}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2873A9DE-E1DD-42D4-AAAD-684C6487C98C}">
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1654,24 +1662,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
       <c r="G3" t="s">
         <v>71</v>
       </c>
@@ -1716,22 +1724,22 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="1"/>
@@ -1753,7 +1761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60450CF1-74A0-43DC-B5C1-C125781275B5}">
   <dimension ref="A3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1769,7 +1777,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D785D3B-C307-4104-99E3-4F6D4489ECE3}">
   <dimension ref="A2:M24"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1780,50 +1788,49 @@
   <sheetData>
     <row r="2" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9">
+      <c r="C3" s="7"/>
+      <c r="D3" s="7">
         <v>915</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12">
+      <c r="D4">
         <v>250</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="10" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="13"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
       <c r="L10" t="s">
         <v>78</v>
       </c>
@@ -1845,14 +1852,9 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A13" s="17" t="s">
+      <c r="A13" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
@@ -1866,22 +1868,22 @@
       <c r="J18" s="4"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.45">
       <c r="J23" s="4"/>
@@ -1909,7 +1911,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{294A87B4-F113-4702-B529-F80FE0DA082D}">
   <dimension ref="A6:M47"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1923,46 +1925,46 @@
       </c>
     </row>
     <row r="45" spans="2:13" ht="14.25" customHeight="1" x14ac:dyDescent="1.1499999999999999">
-      <c r="B45" s="18"/>
-      <c r="C45" s="18"/>
-      <c r="D45" s="18"/>
-      <c r="E45" s="18"/>
-      <c r="F45" s="18"/>
-      <c r="G45" s="18"/>
-      <c r="H45" s="18"/>
-      <c r="I45" s="18"/>
-      <c r="J45" s="18"/>
-      <c r="K45" s="18"/>
-      <c r="L45" s="18"/>
-      <c r="M45" s="18"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="14"/>
+      <c r="L45" s="14"/>
+      <c r="M45" s="14"/>
     </row>
     <row r="46" spans="2:13" ht="14.25" customHeight="1" x14ac:dyDescent="1.1499999999999999">
-      <c r="B46" s="18"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="18"/>
-      <c r="E46" s="18"/>
-      <c r="F46" s="18"/>
-      <c r="G46" s="18"/>
-      <c r="H46" s="18"/>
-      <c r="I46" s="18"/>
-      <c r="J46" s="18"/>
-      <c r="K46" s="18"/>
-      <c r="L46" s="18"/>
-      <c r="M46" s="18"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
+      <c r="L46" s="14"/>
+      <c r="M46" s="14"/>
     </row>
     <row r="47" spans="2:13" ht="14.25" customHeight="1" x14ac:dyDescent="1.1499999999999999">
-      <c r="B47" s="18"/>
-      <c r="C47" s="18"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
-      <c r="F47" s="18"/>
-      <c r="G47" s="18"/>
-      <c r="H47" s="18"/>
-      <c r="I47" s="18"/>
-      <c r="J47" s="18"/>
-      <c r="K47" s="18"/>
-      <c r="L47" s="18"/>
-      <c r="M47" s="18"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="14"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="14"/>
+      <c r="K47" s="14"/>
+      <c r="L47" s="14"/>
+      <c r="M47" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>